<commit_message>
Fix top-rank ordering bug: remove 0.999 score clamp that forged ties among the strongest candidates (then ordered by candidate_id, not quality). Normalize by pool max instead: true ordering, scores in [0,1]. Also remove empty src/rerank package and unused deps (PyYAML, tqdm, scikit-learn). Re-verified: validator passes, eval composite 0.952 unchanged, leak test 0/0/0 unchanged.
</commit_message>
<xml_diff>
--- a/submission_package/the_last_commit.xlsx
+++ b/submission_package/the_last_commit.xlsx
@@ -447,108 +447,108 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CAND_0011687</t>
+          <t>CAND_0046525</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.999</v>
+        <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer, 7.8y; career shows retrieval &amp; ranking; GitHub activity 76; responsive to recruiters (0.89); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Senior Machine Learning Engineer, 6.1y; career shows retrieval &amp; ranking; responsive to recruiters (0.88); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CAND_0018499</t>
+          <t>CAND_0077337</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>0.999</v>
+        <v>0.969616</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, 7.2y; career shows retrieval &amp; ranking; GitHub activity 95; responsive to recruiters (0.61); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Staff Machine Learning Engineer, 7.0y; career shows retrieval &amp; ranking; GitHub activity 68; responsive to recruiters (0.95); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAND_0041669</t>
+          <t>CAND_0018499</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>0.999</v>
+        <v>0.966314</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 8.0y; career shows retrieval &amp; ranking; GitHub activity 71; responsive to recruiters (0.77); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Senior Machine Learning Engineer, 7.2y; career shows retrieval &amp; ranking; GitHub activity 95; responsive to recruiters (0.61); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CAND_0046525</t>
+          <t>CAND_0050454</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>0.999</v>
+        <v>0.960768</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, 6.1y; career shows retrieval &amp; ranking; responsive to recruiters (0.88); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>AI Engineer, 6.8y; career shows retrieval &amp; ranking; responsive to recruiters (0.77). Concern: few remaining concerns; verify recency of hands-on coding.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CAND_0050454</t>
+          <t>CAND_0011687</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>0.999</v>
+        <v>0.95579</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>AI Engineer, 6.8y; career shows retrieval &amp; ranking; responsive to recruiters (0.77). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Senior NLP Engineer, 7.8y; career shows retrieval &amp; ranking; GitHub activity 76; responsive to recruiters (0.89); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CAND_0077337</t>
+          <t>CAND_0041669</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>0.999</v>
+        <v>0.9546829999999999</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, 7.0y; career shows retrieval &amp; ranking; GitHub activity 68; responsive to recruiters (0.95); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Recommendation Systems Engineer, 8.0y; career shows retrieval &amp; ranking; GitHub activity 71; responsive to recruiters (0.77); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>0.993586</v>
+        <v>0.947254</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -580,7 +580,7 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>0.980602</v>
+        <v>0.934875</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>0.975021</v>
+        <v>0.929554</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>0.961277</v>
+        <v>0.916451</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -634,7 +634,7 @@
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>0.960789</v>
+        <v>0.915986</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -652,7 +652,7 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>0.955552</v>
+        <v>0.9109930000000001</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>0.951013</v>
+        <v>0.9066650000000001</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -688,7 +688,7 @@
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>0.950675</v>
+        <v>0.906343</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -706,7 +706,7 @@
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>0.947794</v>
+        <v>0.903596</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -724,7 +724,7 @@
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>0.947693</v>
+        <v>0.903501</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -742,7 +742,7 @@
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>0.947479</v>
+        <v>0.903296</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -760,7 +760,7 @@
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>0.944558</v>
+        <v>0.900511</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>0.943665</v>
+        <v>0.89966</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -796,7 +796,7 @@
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>0.938582</v>
+        <v>0.894814</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>0.937928</v>
+        <v>0.894191</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -832,7 +832,7 @@
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>0.933655</v>
+        <v>0.890117</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>0.933319</v>
+        <v>0.8897969999999999</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -868,7 +868,7 @@
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.889493</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -886,7 +886,7 @@
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>0.930068</v>
+        <v>0.886697</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -904,7 +904,7 @@
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>0.929942</v>
+        <v>0.8865769999999999</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>0.928176</v>
+        <v>0.884894</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -940,7 +940,7 @@
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>0.924234</v>
+        <v>0.881135</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -958,7 +958,7 @@
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>0.922384</v>
+        <v>0.879372</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -976,7 +976,7 @@
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>0.920625</v>
+        <v>0.877695</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>0.918496</v>
+        <v>0.875665</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1012,7 +1012,7 @@
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>0.917965</v>
+        <v>0.875159</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1030,7 +1030,7 @@
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>0.916637</v>
+        <v>0.873892</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>0.913037</v>
+        <v>0.870461</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1066,7 +1066,7 @@
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>0.909647</v>
+        <v>0.867229</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1084,7 +1084,7 @@
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>0.908617</v>
+        <v>0.866247</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>0.906282</v>
+        <v>0.86402</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1120,7 +1120,7 @@
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>0.9032</v>
+        <v>0.861082</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1138,7 +1138,7 @@
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>0.901018</v>
+        <v>0.859002</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1156,7 +1156,7 @@
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>0.900851</v>
+        <v>0.858842</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>0.900795</v>
+        <v>0.858789</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1192,7 +1192,7 @@
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>0.898494</v>
+        <v>0.856596</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1210,7 +1210,7 @@
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>0.898333</v>
+        <v>0.856443</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1228,7 +1228,7 @@
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>0.8982520000000001</v>
+        <v>0.856365</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1246,7 +1246,7 @@
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>0.895964</v>
+        <v>0.854183</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1264,7 +1264,7 @@
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>0.8942290000000001</v>
+        <v>0.85253</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1282,7 +1282,7 @@
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>0.8931210000000001</v>
+        <v>0.851473</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1300,7 +1300,7 @@
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>0.8899860000000001</v>
+        <v>0.848484</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>0.888601</v>
+        <v>0.847164</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1336,7 +1336,7 @@
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>0.887964</v>
+        <v>0.846557</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1354,7 +1354,7 @@
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>0.886276</v>
+        <v>0.844948</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1372,7 +1372,7 @@
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>0.885555</v>
+        <v>0.84426</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>0.874922</v>
+        <v>0.8341229999999999</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>0.8729440000000001</v>
+        <v>0.832237</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -1426,7 +1426,7 @@
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>0.871668</v>
+        <v>0.831021</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -1444,7 +1444,7 @@
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>0.869767</v>
+        <v>0.8292079999999999</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1462,7 +1462,7 @@
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>0.866011</v>
+        <v>0.825628</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1480,7 +1480,7 @@
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>0.863551</v>
+        <v>0.823282</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>0.86312</v>
+        <v>0.822871</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1516,7 +1516,7 @@
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>0.860522</v>
+        <v>0.820395</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -1534,7 +1534,7 @@
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>0.85849</v>
+        <v>0.818458</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -1552,7 +1552,7 @@
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>0.857862</v>
+        <v>0.817858</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>0.857777</v>
+        <v>0.817778</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -1588,7 +1588,7 @@
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>0.855966</v>
+        <v>0.816051</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -1606,7 +1606,7 @@
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>0.854105</v>
+        <v>0.814277</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -1624,7 +1624,7 @@
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>0.853336</v>
+        <v>0.813544</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -1642,7 +1642,7 @@
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>0.850832</v>
+        <v>0.811156</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -1660,7 +1660,7 @@
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>0.850409</v>
+        <v>0.8107529999999999</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -1678,7 +1678,7 @@
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>0.850371</v>
+        <v>0.810717</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -1696,7 +1696,7 @@
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>0.850067</v>
+        <v>0.810427</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -1714,7 +1714,7 @@
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>0.8499719999999999</v>
+        <v>0.8103359999999999</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -1732,7 +1732,7 @@
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>0.848952</v>
+        <v>0.809364</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -1750,7 +1750,7 @@
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>0.848708</v>
+        <v>0.809131</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -1768,7 +1768,7 @@
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>0.845488</v>
+        <v>0.806061</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>0.844201</v>
+        <v>0.804835</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -1804,7 +1804,7 @@
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>0.842025</v>
+        <v>0.80276</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -1822,7 +1822,7 @@
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>0.841653</v>
+        <v>0.802405</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -1840,7 +1840,7 @@
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>0.840275</v>
+        <v>0.801091</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>0.839769</v>
+        <v>0.800609</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -1876,7 +1876,7 @@
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>0.839724</v>
+        <v>0.800566</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -1894,7 +1894,7 @@
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>0.838943</v>
+        <v>0.799821</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -1912,7 +1912,7 @@
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>0.837852</v>
+        <v>0.798781</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>0.836667</v>
+        <v>0.797652</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>0.835759</v>
+        <v>0.796786</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>0.832272</v>
+        <v>0.793462</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -1984,7 +1984,7 @@
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>0.831551</v>
+        <v>0.792774</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -2002,7 +2002,7 @@
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>0.823034</v>
+        <v>0.784655</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -2020,7 +2020,7 @@
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>0.822948</v>
+        <v>0.784573</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -2038,7 +2038,7 @@
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>0.821655</v>
+        <v>0.78334</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -2056,7 +2056,7 @@
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>0.821486</v>
+        <v>0.783179</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -2074,7 +2074,7 @@
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>0.82138</v>
+        <v>0.7830780000000001</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2092,7 +2092,7 @@
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>0.8194900000000001</v>
+        <v>0.7812750000000001</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -2110,7 +2110,7 @@
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>0.818855</v>
+        <v>0.78067</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>0.8186560000000001</v>
+        <v>0.780481</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -2146,7 +2146,7 @@
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>0.818617</v>
+        <v>0.780443</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2164,7 +2164,7 @@
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>0.8176020000000001</v>
+        <v>0.7794759999999999</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2182,7 +2182,7 @@
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>0.817265</v>
+        <v>0.779154</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -2200,7 +2200,7 @@
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>0.816252</v>
+        <v>0.778189</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -2218,7 +2218,7 @@
         <v>99</v>
       </c>
       <c r="C100" t="n">
-        <v>0.815164</v>
+        <v>0.777152</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -2236,7 +2236,7 @@
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>0.813959</v>
+        <v>0.776003</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Upgrade reasoning generator for Stage-4 variation: candidate-specific facts with concrete values (response %, notice days, assessment scores, named employers), rotated sentence skeletons seeded by candidate_id, evidence fact always cited first, and no stat praised and flagged in the same row. 100/100 unique reasonings (was 51 sharing one concern string). Ranking untouched: validator passes, order identical.
</commit_message>
<xml_diff>
--- a/submission_package/the_last_commit.xlsx
+++ b/submission_package/the_last_commit.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, 6.1y; career shows retrieval &amp; ranking; responsive to recruiters (0.88); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>6.1y Senior Machine Learning Engineer; hands-on ranking &amp; re-rank work at Genpact AI; replies to 88% of recruiter messages; based in Pune. Main caveat: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -476,7 +476,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, 7.0y; career shows retrieval &amp; ranking; GitHub activity 68; responsive to recruiters (0.95); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>7.0y Staff Machine Learning Engineer; hands-on retrieval &amp; ranking work at Paytm; active GitHub (score 68); replies to 95% of recruiter messages. Main caveat: average stint is only ~21 months across 4 roles.</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, 7.2y; career shows retrieval &amp; ranking; GitHub activity 95; responsive to recruiters (0.61); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Senior Machine Learning Engineer, 7.2 yrs. Hands-on ranking &amp; re-rank work at Zomato; active GitHub (score 95); decent recruiter response rate (0.61). One flag: little to fault on paper; verify depth in a technical screen.</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>AI Engineer, 6.8y; career shows retrieval &amp; ranking; responsive to recruiters (0.77). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>AI Engineer with 6.8y: hands-on retrieval &amp; ranking work at Rephrase.ai; replies to 77% of recruiter messages; can move on ~30-day notice. Watch-out: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer, 7.8y; career shows retrieval &amp; ranking; GitHub activity 76; responsive to recruiters (0.89); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Senior NLP Engineer, 7.8 yrs. Hands-on recommend &amp; retrieval work at Niramai; replies to 89% of recruiter messages; can move on ~15-day notice. One flag: little to fault on paper; verify depth in a technical screen.</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 8.0y; career shows retrieval &amp; ranking; GitHub activity 71; responsive to recruiters (0.77); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>8.0y Recommendation Systems Engineer; hands-on embedding &amp; ranking work at CRED; Redrob assessment 84 in FAISS; has evaluated rankers with NDCG/MRR/A-B testing. Main caveat: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Search Engineer, 7.6y; career shows retrieval &amp; ranking; GitHub activity 61; responsive to recruiters (0.94); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Search Engineer with 7.6y: hands-on ranking &amp; embedding work at Sarvam AI; active GitHub (score 61); replies to 94% of recruiter messages. Watch-out: little to fault on paper; verify depth in a technical screen.</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AI Engineer, 7.3y; career shows retrieval &amp; ranking; GitHub activity 53; responsive to recruiters (0.78). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>AI Engineer, 7.3 yrs. Hands-on retrieval &amp; ranking work at Google; open to relocation; active GitHub (score 53). One flag: ~70 days since last platform activity.</t>
         </is>
       </c>
     </row>
@@ -602,7 +602,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Applied ML Engineer, 8.0y; career shows retrieval &amp; ranking; evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Applied ML Engineer, 8.0 yrs. Hands-on ranking &amp; recommend work at Freshworks; has evaluated rankers with NDCG/MRR/A-B testing; can move on ~30-day notice. One flag: response rate of 0.42 may slow outreach.</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 7.9y; career shows retrieval &amp; recommend; GitHub activity 69; responsive to recruiters (0.62); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>7.9y Recommendation Systems Engineer; hands-on recommend &amp; embedding work at Wysa; based in Noida; has evaluated rankers with NDCG/MRR/A-B testing. Main caveat: ~105 days since last platform activity.</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Applied ML Engineer, 6.2y; career shows retrieval &amp; ranking; responsive to recruiters (0.82); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>6.2y Applied ML Engineer; hands-on retrieval &amp; ranking work at Zomato; has evaluated rankers with NDCG/MRR/A-B testing; replies to 82% of recruiter messages. Main caveat: ~84 days since last platform activity.</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Senior AI Engineer, 7.8y; career shows retrieval &amp; ranking; GitHub activity 83; responsive to recruiters (0.76); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Senior AI Engineer with 7.8y: hands-on ranking &amp; re-rank work at Netflix; replies to 76% of recruiter messages; Redrob assessment 87 in LoRA. Watch-out: ~77 days since last platform activity.</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, 7.4y; career shows retrieval &amp; ranking; GitHub activity 81; evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>7.4y Senior Data Scientist; hands-on retrieval &amp; ranking work at Sarvam AI; active GitHub (score 81); decent recruiter response rate (0.57). Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>AI Engineer, 6.3y; career shows retrieval &amp; ranking; GitHub activity 70; responsive to recruiters (0.84); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>AI Engineer, 6.3 yrs. Hands-on retrieval &amp; ranking work at Mad Street Den; open to relocation; has evaluated rankers with NDCG/MRR/A-B testing. One flag: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>AI Engineer, 6.4y; career shows retrieval &amp; ranking; responsive to recruiters (0.86); evaluation-metric experience (NDCG/MRR/A-B). Concern: not marked open-to-work.</t>
+          <t>AI Engineer with 6.4y: hands-on retrieval &amp; ranking work at Mad Street Den; Redrob assessment 90 in TensorFlow; has evaluated rankers with NDCG/MRR/A-B testing. Watch-out: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
@@ -728,7 +728,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>NLP Engineer, 6.7y; career shows retrieval &amp; ranking; responsive to recruiters (0.83); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>6.7y NLP Engineer; hands-on semantic search &amp; retrieval work at Rephrase.ai; can move on ~30-day notice; has evaluated rankers with NDCG/MRR/A-B testing. Main caveat: average stint is only ~20 months across 4 roles.</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 6.0y; career shows retrieval &amp; recommend; GitHub activity 43; responsive to recruiters (0.90). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Recommendation Systems Engineer, 6.0y: hands-on recommend &amp; semantic search work at CRED; active GitHub (score 43); replies to 90% of recruiter messages. Concern: little to fault on paper; verify depth in a technical screen.</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Applied ML Engineer, 7.1y; career shows retrieval &amp; ranking; GitHub activity 86; responsive to recruiters (0.61); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>Applied ML Engineer, 7.1 yrs. Hands-on semantic search &amp; retrieval work at Meesho; based in Gurgaon; Redrob assessment 86 in Hugging Face Transformers. One flag: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, 6.5y; career shows retrieval &amp; ranking; GitHub activity 46; responsive to recruiters (0.72); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (120 days).</t>
+          <t>6.5y Senior Data Scientist; hands-on ranking &amp; recommend work at Google; decent recruiter response rate (0.72); based in Noida. Main caveat: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NLP Engineer, 7.4y; career shows retrieval &amp; recommend; GitHub activity 63; responsive to recruiters (0.65). Concern: long notice period (120 days).</t>
+          <t>7.4y NLP Engineer; hands-on retrieval &amp; recommend work at InMobi; decent recruiter response rate (0.65); based in Hyderabad. Main caveat: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer, 8.9y; career shows retrieval &amp; ranking; GitHub activity 67; responsive to recruiters (0.78); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Senior NLP Engineer, 8.9y: hands-on re-rank &amp; retrieval work at Salesforce; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 67). Concern: ~67 days since last platform activity.</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>AI Engineer, 7.7y; career shows retrieval &amp; ranking; responsive to recruiters (0.60); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>AI Engineer with 7.7y: hands-on semantic search &amp; retrieval work at PolicyBazaar; Redrob assessment 85 in LlamaIndex; has evaluated rankers with NDCG/MRR/A-B testing. Watch-out: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>NLP Engineer, 6.5y; career shows retrieval &amp; ranking; GitHub activity 58; responsive to recruiters (0.68). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>NLP Engineer, 6.5 yrs. Hands-on ranking &amp; semantic search work at Haptik; decent recruiter response rate (0.68); can move on ~15-day notice. One flag: ~93 days since last platform activity.</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Junior ML Engineer, 6.1y; career shows retrieval &amp; ranking; responsive to recruiters (0.81). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Junior ML Engineer, 6.1y: hands-on ranking &amp; re-rank work at Aganitha; replies to 81% of recruiter messages; can move on ~30-day notice. Concern: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>AI Engineer, 6.9y; career shows retrieval &amp; ranking; GitHub activity 64; responsive to recruiters (0.81); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>AI Engineer, 6.9 yrs. Hands-on ranking &amp; recommend work at Microsoft; replies to 81% of recruiter messages; can move on ~30-day notice. One flag: average stint is only ~20 months across 4 roles.</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer, 7.8y; career shows retrieval &amp; ranking; GitHub activity 53; responsive to recruiters (0.66); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>7.8y Senior NLP Engineer; hands-on ranking &amp; recommend work at Ola; active GitHub (score 53); decent recruiter response rate (0.66). Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Lead AI Engineer, 6.7y; career shows retrieval &amp; ranking; responsive to recruiters (0.73); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Lead AI Engineer with 6.7y: hands-on retrieval &amp; ranking work at Razorpay; can move on ~30-day notice; open to relocation. Watch-out: little to fault on paper; verify depth in a technical screen.</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 6.8y; career shows retrieval &amp; ranking; GitHub activity 56; responsive to recruiters (0.73); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>6.8y Recommendation Systems Engineer; hands-on ranking &amp; recommend work at Uber; Redrob assessment 90 in Elasticsearch; has evaluated rankers with NDCG/MRR/A-B testing. Main caveat: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>NLP Engineer, 6.8y; career shows retrieval &amp; ranking; responsive to recruiters (0.83); evaluation-metric experience (NDCG/MRR/A-B). Concern: not marked open-to-work.</t>
+          <t>NLP Engineer, 6.8 yrs. Hands-on recommend &amp; retrieval work at Locobuzz; Redrob assessment 81 in Deep Learning; has evaluated rankers with NDCG/MRR/A-B testing. One flag: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, 7.2y; career shows retrieval &amp; ranking; GitHub activity 63; responsive to recruiters (0.60); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (120 days).</t>
+          <t>Machine Learning Engineer with 7.2y: hands-on retrieval &amp; ranking work at Genpact AI; open to relocation; Redrob assessment 85 in RAG. Watch-out: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>AI Research Engineer, 6.0y; career shows retrieval &amp; ranking; responsive to recruiters (0.83). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>AI Research Engineer with 6.0y: hands-on re-rank &amp; recommend work at Yellow.ai; based in Delhi; Redrob assessment 86 in TTS. Watch-out: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Applied ML Engineer, 6.7y; career shows retrieval &amp; ranking; GitHub activity 95; responsive to recruiters (0.72). Concern: long notice period (120 days).</t>
+          <t>Applied ML Engineer, 6.7 yrs. Hands-on relevance &amp; retrieval work at Dream11; Redrob assessment 89 in Time Series; active GitHub (score 95). One flag: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 6.7y; career shows retrieval &amp; ranking; GitHub activity 52; evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Recommendation Systems Engineer with 6.7y: hands-on ranking &amp; recommend work at Zoho; can move on ~30-day notice; open to relocation. Watch-out: average stint is only ~20 months across 4 roles.</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Search Engineer, 6.0y; career shows retrieval &amp; ranking; GitHub activity 46; responsive to recruiters (0.91); evaluation-metric experience (NDCG/MRR/A-B). Concern: not marked open-to-work.</t>
+          <t>Search Engineer with 6.0y: hands-on recommend &amp; retrieval work at Netflix; replies to 91% of recruiter messages; Redrob assessment 86 in FAISS. Watch-out: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 6.6y; career shows retrieval &amp; ranking; GitHub activity 80; responsive to recruiters (0.94). Concern: long notice period (120 days).</t>
+          <t>6.6y Recommendation Systems Engineer; hands-on recommend &amp; retrieval work at Zoho; replies to 94% of recruiter messages; based in Delhi. Main caveat: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Search Engineer, 7.8y; career shows retrieval &amp; ranking; GitHub activity 69; responsive to recruiters (0.70); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (120 days).</t>
+          <t>Search Engineer, 7.8 yrs. Hands-on retrieval &amp; ranking work at CRED; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 69). One flag: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Search Engineer, 7.6y; career shows retrieval &amp; ranking. Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Search Engineer, 7.6 yrs. Hands-on retrieval &amp; semantic search work at Haptik; open to relocation; Redrob assessment 76 in Weaviate. One flag: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, 6.6y; career shows retrieval &amp; ranking; GitHub activity 47; evaluation-metric experience (NDCG/MRR/A-B). Concern: not marked open-to-work.</t>
+          <t>Senior Data Scientist, 6.6 yrs. Hands-on recommend &amp; retrieval work at Flipkart; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 47). One flag: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>NLP Engineer, 7.9y; career shows retrieval &amp; ranking; responsive to recruiters (0.63); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (120 days).</t>
+          <t>7.9y NLP Engineer; hands-on embedding &amp; ranking work at Paytm; decent recruiter response rate (0.63); open to relocation. Main caveat: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Senior Machine Learning Engineer, 8.1y; career shows retrieval &amp; ranking; responsive to recruiters (0.87); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>8.1y Senior Machine Learning Engineer; hands-on retrieval &amp; ranking work at Flipkart; replies to 87% of recruiter messages; can move on ~30-day notice. Main caveat: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Applied ML Engineer, 7.4y; career shows ranking &amp; recommend; responsive to recruiters (0.76); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (120 days).</t>
+          <t>Applied ML Engineer, 7.4y: hands-on embedding &amp; ranking work at Zoho; based in Noida; has evaluated rankers with NDCG/MRR/A-B testing. Concern: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Senior NLP Engineer, 5.2y; career shows retrieval &amp; ranking; responsive to recruiters (0.86); evaluation-metric experience (NDCG/MRR/A-B). Concern: not marked open-to-work.</t>
+          <t>Senior NLP Engineer, 5.2y: hands-on ranking &amp; re-rank work at Netflix; has evaluated rankers with NDCG/MRR/A-B testing; replies to 86% of recruiter messages. Concern: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Applied ML Engineer, 6.6y; career shows retrieval &amp; ranking; GitHub activity 45; responsive to recruiters (0.78); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>6.6y Applied ML Engineer; hands-on embedding &amp; retrieval work at Sarvam AI; active GitHub (score 45); replies to 78% of recruiter messages. Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>AI Engineer, 7.6y; career shows retrieval &amp; ranking; GitHub activity 86; responsive to recruiters (0.62); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>AI Engineer with 7.6y: hands-on relevance &amp; ranking work at upGrad; decent recruiter response rate (0.62); open to relocation. Watch-out: ~70 days since last platform activity.</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Applied ML Engineer, 6.4y; career shows ranking &amp; recommend; responsive to recruiters (0.79); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Applied ML Engineer, 6.4 yrs. Hands-on ranking &amp; embedding work at Aganitha; has evaluated rankers with NDCG/MRR/A-B testing; replies to 79% of recruiter messages. One flag: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>NLP Engineer, 6.6y; career shows ranking &amp; recommend; GitHub activity 72; responsive to recruiters (0.88); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>NLP Engineer with 6.6y: hands-on embedding &amp; ranking work at Aganitha; replies to 88% of recruiter messages; can move on ~30-day notice. Watch-out: ~96 days since last platform activity.</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>AI Engineer, 6.7y; career shows ranking &amp; recommend; responsive to recruiters (0.74); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>AI Engineer, 6.7y: hands-on embedding &amp; ranking work at Vedantu; has evaluated rankers with NDCG/MRR/A-B testing; decent recruiter response rate (0.74). Concern: ~96 days since last platform activity.</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, 5.2y; career shows retrieval &amp; ranking; responsive to recruiters (0.91); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (120 days).</t>
+          <t>Senior Data Scientist, 5.2y: hands-on semantic search &amp; retrieval work at Niramai; based in Noida; has evaluated rankers with NDCG/MRR/A-B testing. Concern: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, 8.6y; career shows retrieval &amp; ranking; GitHub activity 75; responsive to recruiters (0.83); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>8.6y Staff Machine Learning Engineer; hands-on recommend &amp; retrieval work at Yellow.ai; active GitHub (score 75); replies to 83% of recruiter messages. Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 7.7y; career shows retrieval &amp; ranking; GitHub activity 52; evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (120 days).</t>
+          <t>Recommendation Systems Engineer, 7.7 yrs. Hands-on retrieval &amp; ranking work at Wysa; Redrob assessment 84 in Recommendation Systems; has evaluated rankers with NDCG/MRR/A-B testing. One flag: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 6.4y; career shows retrieval &amp; ranking; GitHub activity 90; responsive to recruiters (0.64). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Recommendation Systems Engineer, 6.4y: hands-on recommend &amp; relevance work at CRED; decent recruiter response rate (0.64); based in Chennai. Concern: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, 6.9y; career shows retrieval &amp; ranking; GitHub activity 50; responsive to recruiters (0.65); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>6.9y Machine Learning Engineer; hands-on recommend &amp; embedding work at Rephrase.ai; Redrob assessment 90 in Image Classification; has evaluated rankers with NDCG/MRR/A-B testing. Main caveat: ~106 days since last platform activity.</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Applied ML Engineer, 5.0y; career shows retrieval &amp; ranking; GitHub activity 80; responsive to recruiters (0.84); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (120 days).</t>
+          <t>Applied ML Engineer with 5.0y: hands-on recommend &amp; embedding work at upGrad; replies to 84% of recruiter messages; based in Hyderabad. Watch-out: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 7.7y; career shows ranking &amp; recommend; GitHub activity 92; responsive to recruiters (0.72); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Recommendation Systems Engineer, 7.7y: hands-on embedding &amp; ranking work at Nykaa; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 92). Concern: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Junior ML Engineer, 6.4y; career shows retrieval &amp; ranking; responsive to recruiters (0.81). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>6.4y Junior ML Engineer; hands-on ranking &amp; re-rank work at Sarvam AI; replies to 81% of recruiter messages; open to relocation. Main caveat: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Data Scientist, 6.7y; career shows retrieval &amp; ranking; responsive to recruiters (0.80). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Data Scientist with 6.7y: hands-on ranking &amp; re-rank work at Rephrase.ai; replies to 80% of recruiter messages; can move on ~30-day notice. Watch-out: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Applied ML Engineer, 6.8y; career shows retrieval &amp; ranking; GitHub activity 48. Concern: not marked open-to-work.</t>
+          <t>Applied ML Engineer, 6.8y: hands-on ranking &amp; semantic search work at Zoho; active GitHub (score 48); can move on ~30-day notice. Concern: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>ML Engineer, 6.9y; career shows ranking &amp; re-rank; responsive to recruiters (0.82). Concern: long notice period (90 days).</t>
+          <t>6.9y ML Engineer; hands-on ranking &amp; re-rank work at Glance; replies to 82% of recruiter messages; based in Bangalore. Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>NLP Engineer, 5.9y; career shows retrieval &amp; ranking; GitHub activity 65; responsive to recruiters (0.82). Concern: long notice period (120 days).</t>
+          <t>NLP Engineer, 5.9y: hands-on retrieval &amp; recommend work at Rephrase.ai; active GitHub (score 65); replies to 82% of recruiter messages. Concern: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>AI Research Engineer, 6.3y; career shows retrieval &amp; ranking; responsive to recruiters (0.79). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>AI Research Engineer, 6.3 yrs. Hands-on recommend &amp; ranking work at Krutrim; replies to 79% of recruiter messages; based in Gurgaon. One flag: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, 6.3y; career shows retrieval &amp; ranking; GitHub activity 51; responsive to recruiters (0.86); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Machine Learning Engineer with 6.3y: hands-on embedding &amp; ranking work at Meta; replies to 86% of recruiter messages; Redrob assessment 80 in pgvector. Watch-out: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 6.6y; career shows retrieval &amp; ranking; GitHub activity 94; responsive to recruiters (0.79). Concern: long notice period (90 days).</t>
+          <t>Recommendation Systems Engineer with 6.6y: hands-on recommend &amp; retrieval work at Saarthi.ai; open to relocation; active GitHub (score 94). Watch-out: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1574,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Applied ML Engineer, 5.2y; career shows retrieval &amp; ranking; GitHub activity 62; evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Applied ML Engineer, 5.2y: hands-on ranking &amp; embedding work at Freshworks; active GitHub (score 62); can move on ~30-day notice. Concern: average stint is only ~20 months across 3 roles.</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Search Engineer, 7.3y; career shows retrieval &amp; ranking; evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>Search Engineer, 7.3y: hands-on ranking &amp; recommend work at Unacademy; has evaluated rankers with NDCG/MRR/A-B testing; open to relocation. Concern: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Senior Applied Scientist, 16.2y; career shows retrieval &amp; ranking; GitHub activity 78; responsive to recruiters (0.81); evaluation-metric experience (NDCG/MRR/A-B). Concern: 16.2y experience is outside the 5-9y target band.</t>
+          <t>Senior Applied Scientist with 16.2y: hands-on ranking &amp; re-rank work at Meta; open to relocation; Redrob assessment 96 in Fine-tuning LLMs. Watch-out: 16.2y experience falls outside the JD's 5-9y band.</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 6.0y; career shows retrieval &amp; ranking; responsive to recruiters (0.91); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Recommendation Systems Engineer, 6.0 yrs. Hands-on recommend &amp; relevance work at Swiggy; Redrob assessment 75 in MLflow; has evaluated rankers with NDCG/MRR/A-B testing. One flag: average stint is only ~18 months across 4 roles.</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Search Engineer, 7.2y; career shows retrieval &amp; ranking; GitHub activity 83; evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (120 days).</t>
+          <t>7.2y Search Engineer; hands-on embedding &amp; retrieval work at Google; open to relocation; Redrob assessment 89 in Embeddings. Main caveat: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>AI Research Engineer, 6.9y; career shows retrieval &amp; ranking; responsive to recruiters (0.84). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>AI Research Engineer, 6.9 yrs. Hands-on recommend &amp; ranking work at Wipro; Redrob assessment 82 in Speech Recognition; replies to 84% of recruiter messages. One flag: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, 7.6y; career shows retrieval &amp; ranking; responsive to recruiters (0.67); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Senior Data Scientist, 7.6y: hands-on machine learning &amp; ranking work at Amazon; has evaluated rankers with NDCG/MRR/A-B testing; decent recruiter response rate (0.67). Concern: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, 5.3y; career shows retrieval &amp; ranking; evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Senior Data Scientist, 5.3y: hands-on embedding &amp; ranking work at Netflix; Redrob assessment 87 in pgvector; has evaluated rankers with NDCG/MRR/A-B testing. Concern: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>NLP Engineer, 7.7y; career shows retrieval &amp; ranking; evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>7.7y NLP Engineer; hands-on embedding &amp; ranking work at Dream11; has evaluated rankers with NDCG/MRR/A-B testing; open to relocation. Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, 6.5y; career shows retrieval &amp; ranking; GitHub activity 79; responsive to recruiters (0.67); evaluation-metric experience (NDCG/MRR/A-B). Concern: not marked open-to-work.</t>
+          <t>6.5y Senior Data Scientist; hands-on machine learning &amp; ranking work at Flipkart; Redrob assessment 83 in YOLO; has evaluated rankers with NDCG/MRR/A-B testing. Main caveat: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
@@ -1754,7 +1754,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Senior AI Engineer, 5.9y; career shows retrieval &amp; ranking; GitHub activity 97; responsive to recruiters (0.80); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>5.9y Senior AI Engineer; hands-on ranking &amp; re-rank work at Apple; active GitHub (score 97); replies to 80% of recruiter messages. Main caveat: little to fault on paper; verify depth in a technical screen.</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, 7.0y; career shows retrieval &amp; ranking; GitHub activity 90; evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>7.0y Senior Data Scientist; hands-on ranking &amp; recommend work at Microsoft; active GitHub (score 90); open to relocation. Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Search Engineer, 7.8y; career shows retrieval &amp; ranking; responsive to recruiters (0.63); evaluation-metric experience (NDCG/MRR/A-B). Concern: not marked open-to-work.</t>
+          <t>7.8y Search Engineer; hands-on recommend &amp; retrieval work at Nykaa; decent recruiter response rate (0.63); based in Chennai. Main caveat: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, 7.1y; career shows ranking &amp; recommend. Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Machine Learning Engineer, 7.1y: hands-on ranking &amp; relevance work at Unacademy; can move on ~30-day notice. Concern: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>NLP Engineer, 5.4y; career shows ranking &amp; recommend; GitHub activity 78; responsive to recruiters (0.83); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>5.4y NLP Engineer; hands-on embedding &amp; ranking work at Glance; open to relocation; Redrob assessment 89 in QLoRA. Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Senior AI Engineer, 7.9y; career shows retrieval &amp; ranking; responsive to recruiters (0.79); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Senior AI Engineer, 7.9 yrs. Hands-on ranking &amp; relevance work at Meta; Redrob assessment 90 in scikit-learn; has evaluated rankers with NDCG/MRR/A-B testing. One flag: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -1862,7 +1862,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, 5.1y; career shows retrieval &amp; ranking; responsive to recruiters (0.60); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>Machine Learning Engineer with 5.1y: hands-on embedding &amp; ranking work at BYJU'S; Redrob assessment 89 in Object Detection; has evaluated rankers with NDCG/MRR/A-B testing. Watch-out: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Applied ML Engineer, 7.4y; career shows retrieval &amp; ranking; GitHub activity 51; evaluation-metric experience (NDCG/MRR/A-B). Concern: not marked open-to-work.</t>
+          <t>Applied ML Engineer, 7.4y: hands-on ranking &amp; recommend work at Krutrim; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 51). Concern: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Applied ML Engineer, 6.0y; career shows ranking &amp; recommend; GitHub activity 86; responsive to recruiters (0.67); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>Applied ML Engineer, 6.0y: hands-on embedding &amp; ranking work at Freshworks; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 86). Concern: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, 5.3y; career shows retrieval &amp; ranking; GitHub activity 82; responsive to recruiters (0.66). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Senior Data Scientist, 5.3y: hands-on retrieval &amp; ranking work at Razorpay; active GitHub (score 82); decent recruiter response rate (0.66). Concern: average stint is only ~21 months across 3 roles.</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, 8.0y; career shows retrieval &amp; ranking; GitHub activity 45; responsive to recruiters (0.87); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>8.0y Staff Machine Learning Engineer; hands-on ranking &amp; relevance work at LinkedIn; replies to 87% of recruiter messages; can move on ~30-day notice. Main caveat: ~77 days since last platform activity.</t>
         </is>
       </c>
     </row>
@@ -1952,7 +1952,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 4.8y; career shows retrieval &amp; ranking; evaluation-metric experience (NDCG/MRR/A-B). Concern: 4.8y experience is outside the 5-9y target band.</t>
+          <t>Recommendation Systems Engineer, 4.8y: hands-on retrieval &amp; ranking work at Zomato; has evaluated rankers with NDCG/MRR/A-B testing; based in Chennai. Concern: 4.8y experience falls outside the JD's 5-9y band.</t>
         </is>
       </c>
     </row>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, 7.3y; career shows ranking &amp; recommend; GitHub activity 43; responsive to recruiters (0.87); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>Machine Learning Engineer, 7.3y: hands-on relevance &amp; machine learning work at Freshworks; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 43). Concern: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Junior ML Engineer, 7.0y; career shows ranking &amp; re-rank; responsive to recruiters (0.81). Concern: long notice period (90 days).</t>
+          <t>Junior ML Engineer, 7.0 yrs. Hands-on re-rank &amp; recommend work at PhonePe; replies to 81% of recruiter messages; based in Bangalore. One flag: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>ML Engineer, 4.4y; career shows retrieval &amp; ranking; responsive to recruiters (0.89). Concern: 4.4y experience is outside the 5-9y target band.</t>
+          <t>ML Engineer, 4.4 yrs. Hands-on ranking &amp; re-rank work at Glance; replies to 89% of recruiter messages; Redrob assessment 78 in Information Retrieval. One flag: 4.4y experience falls outside the JD's 5-9y band.</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 5.9y; career shows ranking &amp; recommend; GitHub activity 94; responsive to recruiters (0.63). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Recommendation Systems Engineer, 5.9 yrs. Hands-on ranking &amp; recommend work at Microsoft; Redrob assessment 90 in Pinecone; active GitHub (score 94). One flag: ~88 days since last platform activity.</t>
         </is>
       </c>
     </row>
@@ -2042,7 +2042,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Search Engineer, 7.8y; career shows retrieval &amp; ranking; evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>7.8y Search Engineer; hands-on ranking &amp; recommend work at Genpact AI; has evaluated rankers with NDCG/MRR/A-B testing; decent recruiter response rate (0.58). Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -2060,7 +2060,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>NLP Engineer, 6.9y; career shows ranking &amp; recommend; GitHub activity 85; responsive to recruiters (0.84). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>NLP Engineer, 6.9 yrs. Hands-on nlp &amp; ranking work at Ola; Redrob assessment 92 in BM25; active GitHub (score 85). One flag: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Data Scientist, 6.9y; career shows retrieval &amp; ranking; responsive to recruiters (0.73). Concern: long notice period (90 days).</t>
+          <t>Data Scientist with 6.9y: hands-on ranking &amp; re-rank work at upGrad; decent recruiter response rate (0.73); open to relocation. Watch-out: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, 5.7y; career shows ranking &amp; recommend; evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>Machine Learning Engineer with 5.7y: hands-on embedding &amp; relevance work at Haptik; based in Bangalore; Redrob assessment 83 in pgvector. Watch-out: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
@@ -2114,7 +2114,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, 4.6y; career shows ranking &amp; recommend; GitHub activity 56; responsive to recruiters (0.88); evaluation-metric experience (NDCG/MRR/A-B). Concern: 4.6y experience is outside the 5-9y target band.</t>
+          <t>Machine Learning Engineer, 4.6 yrs. Hands-on embedding &amp; ranking work at Krutrim; can move on ~15-day notice; has evaluated rankers with NDCG/MRR/A-B testing. One flag: 4.6y experience falls outside the JD's 5-9y band.</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Machine Learning Engineer, 6.0y; career shows retrieval &amp; ranking; GitHub activity 66. Concern: long notice period (90 days).</t>
+          <t>Machine Learning Engineer with 6.0y: hands-on retrieval &amp; ranking work at Razorpay; active GitHub (score 66). Watch-out: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer, 8.8y; career shows retrieval &amp; ranking; responsive to recruiters (0.66); evaluation-metric experience (NDCG/MRR/A-B). Concern: not marked open-to-work.</t>
+          <t>Staff Machine Learning Engineer with 8.8y: hands-on retrieval &amp; ranking work at Salesforce; decent recruiter response rate (0.66); can move on ~0-day notice. Watch-out: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>ML Engineer, 5.0y; career shows retrieval &amp; ranking. Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>ML Engineer with 5.0y: hands-on recommend &amp; ranking work at Meesho; decent recruiter response rate (0.55); based in Pune. Watch-out: average stint is only ~20 months across 3 roles.</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Senior Data Scientist, 5.7y; career shows retrieval &amp; ranking; responsive to recruiters (0.77); evaluation-metric experience (NDCG/MRR/A-B). Concern: long notice period (90 days).</t>
+          <t>Senior Data Scientist, 5.7 yrs. Hands-on retrieval &amp; embedding work at Rephrase.ai; Redrob assessment 90 in Haystack; has evaluated rankers with NDCG/MRR/A-B testing. One flag: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Recommendation Systems Engineer, 6.5y; career shows retrieval &amp; ranking; responsive to recruiters (0.66); evaluation-metric experience (NDCG/MRR/A-B). Concern: few remaining concerns; verify recency of hands-on coding.</t>
+          <t>6.5y Recommendation Systems Engineer; hands-on recommend &amp; embedding work at PhonePe; decent recruiter response rate (0.66); can move on ~15-day notice. Main caveat: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>NLP Engineer, 5.2y; career shows retrieval &amp; ranking; GitHub activity 65; evaluation-metric experience (NDCG/MRR/A-B). Concern: not marked open-to-work.</t>
+          <t>NLP Engineer, 5.2y: hands-on ranking &amp; recommend work at Krutrim; active GitHub (score 65); based in Chennai. Concern: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
@@ -2240,7 +2240,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>AI Engineer, 7.2y; career shows ranking &amp; recommend; evaluation-metric experience (NDCG/MRR/A-B). Concern: not marked open-to-work.</t>
+          <t>AI Engineer with 7.2y: hands-on ranking &amp; recommend work at Vedantu; based in Gurgaon; Redrob assessment 78 in pgvector. Watch-out: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync packaged XLSX with wrapped-reasoning version (matches portal upload)
</commit_message>
<xml_diff>
--- a/submission_package/the_last_commit.xlsx
+++ b/submission_package/the_last_commit.xlsx
@@ -16,14 +16,19 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000000"/>
+  </numFmts>
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +51,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -418,33 +428,33 @@
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
     <col width="110" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>candidate_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>rank</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>score</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>reasoning</t>
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>CAND_0046525</t>
@@ -453,16 +463,16 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>6.1y Senior Machine Learning Engineer; hands-on ranking &amp; re-rank work at Genpact AI; replies to 88% of recruiter messages; based in Pune. Main caveat: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>CAND_0077337</t>
@@ -471,16 +481,16 @@
       <c r="B3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="2" t="n">
         <v>0.969616</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>7.0y Staff Machine Learning Engineer; hands-on retrieval &amp; ranking work at Paytm; active GitHub (score 68); replies to 95% of recruiter messages. Main caveat: average stint is only ~21 months across 4 roles.</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
           <t>CAND_0018499</t>
@@ -489,16 +499,16 @@
       <c r="B4" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="2" t="n">
         <v>0.966314</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Senior Machine Learning Engineer, 7.2 yrs. Hands-on ranking &amp; re-rank work at Zomato; active GitHub (score 95); decent recruiter response rate (0.61). One flag: little to fault on paper; verify depth in a technical screen.</t>
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
           <t>CAND_0050454</t>
@@ -507,16 +517,16 @@
       <c r="B5" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="2" t="n">
         <v>0.960768</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>AI Engineer with 6.8y: hands-on retrieval &amp; ranking work at Rephrase.ai; replies to 77% of recruiter messages; can move on ~30-day notice. Watch-out: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
           <t>CAND_0011687</t>
@@ -525,16 +535,16 @@
       <c r="B6" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="2" t="n">
         <v>0.95579</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Senior NLP Engineer, 7.8 yrs. Hands-on recommend &amp; retrieval work at Niramai; replies to 89% of recruiter messages; can move on ~15-day notice. One flag: little to fault on paper; verify depth in a technical screen.</t>
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" t="inlineStr">
         <is>
           <t>CAND_0041669</t>
@@ -543,16 +553,16 @@
       <c r="B7" t="n">
         <v>6</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="2" t="n">
         <v>0.9546829999999999</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>8.0y Recommendation Systems Engineer; hands-on embedding &amp; ranking work at CRED; Redrob assessment 84 in FAISS; has evaluated rankers with NDCG/MRR/A-B testing. Main caveat: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" t="inlineStr">
         <is>
           <t>CAND_0064326</t>
@@ -561,16 +571,16 @@
       <c r="B8" t="n">
         <v>7</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="2" t="n">
         <v>0.947254</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Search Engineer with 7.6y: hands-on ranking &amp; embedding work at Sarvam AI; active GitHub (score 61); replies to 94% of recruiter messages. Watch-out: little to fault on paper; verify depth in a technical screen.</t>
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>CAND_0062247</t>
@@ -579,16 +589,16 @@
       <c r="B9" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="2" t="n">
         <v>0.934875</v>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>AI Engineer, 7.3 yrs. Hands-on retrieval &amp; ranking work at Google; open to relocation; active GitHub (score 53). One flag: ~70 days since last platform activity.</t>
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="42" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>CAND_0068811</t>
@@ -597,16 +607,16 @@
       <c r="B10" t="n">
         <v>9</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="2" t="n">
         <v>0.929554</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Applied ML Engineer, 8.0 yrs. Hands-on ranking &amp; recommend work at Freshworks; has evaluated rankers with NDCG/MRR/A-B testing; can move on ~30-day notice. One flag: response rate of 0.42 may slow outreach.</t>
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="42" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>CAND_0007009</t>
@@ -615,16 +625,16 @@
       <c r="B11" t="n">
         <v>10</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="2" t="n">
         <v>0.916451</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>7.9y Recommendation Systems Engineer; hands-on recommend &amp; embedding work at Wysa; based in Noida; has evaluated rankers with NDCG/MRR/A-B testing. Main caveat: ~105 days since last platform activity.</t>
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="42" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
           <t>CAND_0075249</t>
@@ -633,16 +643,16 @@
       <c r="B12" t="n">
         <v>11</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="2" t="n">
         <v>0.915986</v>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>6.2y Applied ML Engineer; hands-on retrieval &amp; ranking work at Zomato; has evaluated rankers with NDCG/MRR/A-B testing; replies to 82% of recruiter messages. Main caveat: ~84 days since last platform activity.</t>
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="42" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
           <t>CAND_0071974</t>
@@ -651,16 +661,16 @@
       <c r="B13" t="n">
         <v>12</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" s="2" t="n">
         <v>0.9109930000000001</v>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Senior AI Engineer with 7.8y: hands-on ranking &amp; re-rank work at Netflix; replies to 76% of recruiter messages; Redrob assessment 87 in LoRA. Watch-out: ~77 days since last platform activity.</t>
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="42" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>CAND_0005649</t>
@@ -669,16 +679,16 @@
       <c r="B14" t="n">
         <v>13</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="2" t="n">
         <v>0.9066650000000001</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>7.4y Senior Data Scientist; hands-on retrieval &amp; ranking work at Sarvam AI; active GitHub (score 81); decent recruiter response rate (0.57). Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="42" customHeight="1">
       <c r="A15" t="inlineStr">
         <is>
           <t>CAND_0044883</t>
@@ -687,16 +697,16 @@
       <c r="B15" t="n">
         <v>14</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="2" t="n">
         <v>0.906343</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>AI Engineer, 6.3 yrs. Hands-on retrieval &amp; ranking work at Mad Street Den; open to relocation; has evaluated rankers with NDCG/MRR/A-B testing. One flag: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="42" customHeight="1">
       <c r="A16" t="inlineStr">
         <is>
           <t>CAND_0060054</t>
@@ -705,16 +715,16 @@
       <c r="B16" t="n">
         <v>15</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" s="2" t="n">
         <v>0.903596</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>AI Engineer with 6.4y: hands-on retrieval &amp; ranking work at Mad Street Den; Redrob assessment 90 in TensorFlow; has evaluated rankers with NDCG/MRR/A-B testing. Watch-out: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="42" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
           <t>CAND_0010685</t>
@@ -723,16 +733,16 @@
       <c r="B17" t="n">
         <v>16</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="2" t="n">
         <v>0.903501</v>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>6.7y NLP Engineer; hands-on semantic search &amp; retrieval work at Rephrase.ai; can move on ~30-day notice; has evaluated rankers with NDCG/MRR/A-B testing. Main caveat: average stint is only ~20 months across 4 roles.</t>
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="42" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
           <t>CAND_0036184</t>
@@ -741,16 +751,16 @@
       <c r="B18" t="n">
         <v>17</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" s="2" t="n">
         <v>0.903296</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Recommendation Systems Engineer, 6.0y: hands-on recommend &amp; semantic search work at CRED; active GitHub (score 43); replies to 90% of recruiter messages. Concern: little to fault on paper; verify depth in a technical screen.</t>
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="42" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
           <t>CAND_0039383</t>
@@ -759,16 +769,16 @@
       <c r="B19" t="n">
         <v>18</v>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" s="2" t="n">
         <v>0.900511</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>Applied ML Engineer, 7.1 yrs. Hands-on semantic search &amp; retrieval work at Meesho; based in Gurgaon; Redrob assessment 86 in Hugging Face Transformers. One flag: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="42" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
           <t>CAND_0010257</t>
@@ -777,16 +787,16 @@
       <c r="B20" t="n">
         <v>19</v>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" s="2" t="n">
         <v>0.89966</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>6.5y Senior Data Scientist; hands-on ranking &amp; recommend work at Google; decent recruiter response rate (0.72); based in Noida. Main caveat: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="42" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
           <t>CAND_0027801</t>
@@ -795,16 +805,16 @@
       <c r="B21" t="n">
         <v>20</v>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" s="2" t="n">
         <v>0.894814</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>7.4y NLP Engineer; hands-on retrieval &amp; recommend work at InMobi; decent recruiter response rate (0.65); based in Hyderabad. Main caveat: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="42" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
           <t>CAND_0046064</t>
@@ -813,16 +823,16 @@
       <c r="B22" t="n">
         <v>21</v>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" s="2" t="n">
         <v>0.894191</v>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Senior NLP Engineer, 8.9y: hands-on re-rank &amp; retrieval work at Salesforce; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 67). Concern: ~67 days since last platform activity.</t>
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="42" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
           <t>CAND_0044222</t>
@@ -831,16 +841,16 @@
       <c r="B23" t="n">
         <v>22</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" s="2" t="n">
         <v>0.890117</v>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>AI Engineer with 7.7y: hands-on semantic search &amp; retrieval work at PolicyBazaar; Redrob assessment 85 in LlamaIndex; has evaluated rankers with NDCG/MRR/A-B testing. Watch-out: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="42" customHeight="1">
       <c r="A24" t="inlineStr">
         <is>
           <t>CAND_0027691</t>
@@ -849,16 +859,16 @@
       <c r="B24" t="n">
         <v>23</v>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" s="2" t="n">
         <v>0.8897969999999999</v>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>NLP Engineer, 6.5 yrs. Hands-on ranking &amp; semantic search work at Haptik; decent recruiter response rate (0.68); can move on ~15-day notice. One flag: ~93 days since last platform activity.</t>
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="42" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
           <t>CAND_0043860</t>
@@ -867,16 +877,16 @@
       <c r="B25" t="n">
         <v>24</v>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" s="2" t="n">
         <v>0.889493</v>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>Junior ML Engineer, 6.1y: hands-on ranking &amp; re-rank work at Aganitha; replies to 81% of recruiter messages; can move on ~30-day notice. Concern: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="42" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
           <t>CAND_0079387</t>
@@ -885,16 +895,16 @@
       <c r="B26" t="n">
         <v>25</v>
       </c>
-      <c r="C26" t="n">
+      <c r="C26" s="2" t="n">
         <v>0.886697</v>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>AI Engineer, 6.9 yrs. Hands-on ranking &amp; recommend work at Microsoft; replies to 81% of recruiter messages; can move on ~30-day notice. One flag: average stint is only ~20 months across 4 roles.</t>
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="42" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
           <t>CAND_0008425</t>
@@ -903,16 +913,16 @@
       <c r="B27" t="n">
         <v>26</v>
       </c>
-      <c r="C27" t="n">
+      <c r="C27" s="2" t="n">
         <v>0.8865769999999999</v>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>7.8y Senior NLP Engineer; hands-on ranking &amp; recommend work at Ola; active GitHub (score 53); decent recruiter response rate (0.66). Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="42" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
           <t>CAND_0081846</t>
@@ -921,16 +931,16 @@
       <c r="B28" t="n">
         <v>27</v>
       </c>
-      <c r="C28" t="n">
+      <c r="C28" s="2" t="n">
         <v>0.884894</v>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>Lead AI Engineer with 6.7y: hands-on retrieval &amp; ranking work at Razorpay; can move on ~30-day notice; open to relocation. Watch-out: little to fault on paper; verify depth in a technical screen.</t>
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="42" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
           <t>CAND_0018549</t>
@@ -939,16 +949,16 @@
       <c r="B29" t="n">
         <v>28</v>
       </c>
-      <c r="C29" t="n">
+      <c r="C29" s="2" t="n">
         <v>0.881135</v>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>6.8y Recommendation Systems Engineer; hands-on ranking &amp; recommend work at Uber; Redrob assessment 90 in Elasticsearch; has evaluated rankers with NDCG/MRR/A-B testing. Main caveat: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="42" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
           <t>CAND_0057563</t>
@@ -957,16 +967,16 @@
       <c r="B30" t="n">
         <v>29</v>
       </c>
-      <c r="C30" t="n">
+      <c r="C30" s="2" t="n">
         <v>0.879372</v>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>NLP Engineer, 6.8 yrs. Hands-on recommend &amp; retrieval work at Locobuzz; Redrob assessment 81 in Deep Learning; has evaluated rankers with NDCG/MRR/A-B testing. One flag: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="42" customHeight="1">
       <c r="A31" t="inlineStr">
         <is>
           <t>CAND_0070398</t>
@@ -975,16 +985,16 @@
       <c r="B31" t="n">
         <v>30</v>
       </c>
-      <c r="C31" t="n">
+      <c r="C31" s="2" t="n">
         <v>0.877695</v>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>Machine Learning Engineer with 7.2y: hands-on retrieval &amp; ranking work at Genpact AI; open to relocation; Redrob assessment 85 in RAG. Watch-out: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="42" customHeight="1">
       <c r="A32" t="inlineStr">
         <is>
           <t>CAND_0004402</t>
@@ -993,16 +1003,16 @@
       <c r="B32" t="n">
         <v>31</v>
       </c>
-      <c r="C32" t="n">
+      <c r="C32" s="2" t="n">
         <v>0.875665</v>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>AI Research Engineer with 6.0y: hands-on re-rank &amp; recommend work at Yellow.ai; based in Delhi; Redrob assessment 86 in TTS. Watch-out: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="42" customHeight="1">
       <c r="A33" t="inlineStr">
         <is>
           <t>CAND_0016163</t>
@@ -1011,16 +1021,16 @@
       <c r="B33" t="n">
         <v>32</v>
       </c>
-      <c r="C33" t="n">
+      <c r="C33" s="2" t="n">
         <v>0.875159</v>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>Applied ML Engineer, 6.7 yrs. Hands-on relevance &amp; retrieval work at Dream11; Redrob assessment 89 in Time Series; active GitHub (score 95). One flag: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="42" customHeight="1">
       <c r="A34" t="inlineStr">
         <is>
           <t>CAND_0041610</t>
@@ -1029,16 +1039,16 @@
       <c r="B34" t="n">
         <v>33</v>
       </c>
-      <c r="C34" t="n">
+      <c r="C34" s="2" t="n">
         <v>0.873892</v>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>Recommendation Systems Engineer with 6.7y: hands-on ranking &amp; recommend work at Zoho; can move on ~30-day notice; open to relocation. Watch-out: average stint is only ~20 months across 4 roles.</t>
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="42" customHeight="1">
       <c r="A35" t="inlineStr">
         <is>
           <t>CAND_0081686</t>
@@ -1047,16 +1057,16 @@
       <c r="B35" t="n">
         <v>34</v>
       </c>
-      <c r="C35" t="n">
+      <c r="C35" s="2" t="n">
         <v>0.870461</v>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>Search Engineer with 6.0y: hands-on recommend &amp; retrieval work at Netflix; replies to 91% of recruiter messages; Redrob assessment 86 in FAISS. Watch-out: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="42" customHeight="1">
       <c r="A36" t="inlineStr">
         <is>
           <t>CAND_0061265</t>
@@ -1065,16 +1075,16 @@
       <c r="B36" t="n">
         <v>35</v>
       </c>
-      <c r="C36" t="n">
+      <c r="C36" s="2" t="n">
         <v>0.867229</v>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>6.6y Recommendation Systems Engineer; hands-on recommend &amp; retrieval work at Zoho; replies to 94% of recruiter messages; based in Delhi. Main caveat: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="42" customHeight="1">
       <c r="A37" t="inlineStr">
         <is>
           <t>CAND_0083307</t>
@@ -1083,16 +1093,16 @@
       <c r="B37" t="n">
         <v>36</v>
       </c>
-      <c r="C37" t="n">
+      <c r="C37" s="2" t="n">
         <v>0.866247</v>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>Search Engineer, 7.8 yrs. Hands-on retrieval &amp; ranking work at CRED; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 69). One flag: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="42" customHeight="1">
       <c r="A38" t="inlineStr">
         <is>
           <t>CAND_0076251</t>
@@ -1101,16 +1111,16 @@
       <c r="B38" t="n">
         <v>37</v>
       </c>
-      <c r="C38" t="n">
+      <c r="C38" s="2" t="n">
         <v>0.86402</v>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>Search Engineer, 7.6 yrs. Hands-on retrieval &amp; semantic search work at Haptik; open to relocation; Redrob assessment 76 in Weaviate. One flag: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="42" customHeight="1">
       <c r="A39" t="inlineStr">
         <is>
           <t>CAND_0044855</t>
@@ -1119,16 +1129,16 @@
       <c r="B39" t="n">
         <v>38</v>
       </c>
-      <c r="C39" t="n">
+      <c r="C39" s="2" t="n">
         <v>0.861082</v>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>Senior Data Scientist, 6.6 yrs. Hands-on recommend &amp; retrieval work at Flipkart; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 47). One flag: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="42" customHeight="1">
       <c r="A40" t="inlineStr">
         <is>
           <t>CAND_0006557</t>
@@ -1137,16 +1147,16 @@
       <c r="B40" t="n">
         <v>39</v>
       </c>
-      <c r="C40" t="n">
+      <c r="C40" s="2" t="n">
         <v>0.859002</v>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>7.9y NLP Engineer; hands-on embedding &amp; ranking work at Paytm; decent recruiter response rate (0.63); open to relocation. Main caveat: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="42" customHeight="1">
       <c r="A41" t="inlineStr">
         <is>
           <t>CAND_0055905</t>
@@ -1155,16 +1165,16 @@
       <c r="B41" t="n">
         <v>40</v>
       </c>
-      <c r="C41" t="n">
+      <c r="C41" s="2" t="n">
         <v>0.858842</v>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>8.1y Senior Machine Learning Engineer; hands-on retrieval &amp; ranking work at Flipkart; replies to 87% of recruiter messages; can move on ~30-day notice. Main caveat: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="42" customHeight="1">
       <c r="A42" t="inlineStr">
         <is>
           <t>CAND_0007412</t>
@@ -1173,16 +1183,16 @@
       <c r="B42" t="n">
         <v>41</v>
       </c>
-      <c r="C42" t="n">
+      <c r="C42" s="2" t="n">
         <v>0.858789</v>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>Applied ML Engineer, 7.4y: hands-on embedding &amp; ranking work at Zoho; based in Noida; has evaluated rankers with NDCG/MRR/A-B testing. Concern: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="42" customHeight="1">
       <c r="A43" t="inlineStr">
         <is>
           <t>CAND_0005260</t>
@@ -1191,16 +1201,16 @@
       <c r="B43" t="n">
         <v>42</v>
       </c>
-      <c r="C43" t="n">
+      <c r="C43" s="2" t="n">
         <v>0.856596</v>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>Senior NLP Engineer, 5.2y: hands-on ranking &amp; re-rank work at Netflix; has evaluated rankers with NDCG/MRR/A-B testing; replies to 86% of recruiter messages. Concern: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="42" customHeight="1">
       <c r="A44" t="inlineStr">
         <is>
           <t>CAND_0069905</t>
@@ -1209,16 +1219,16 @@
       <c r="B44" t="n">
         <v>43</v>
       </c>
-      <c r="C44" t="n">
+      <c r="C44" s="2" t="n">
         <v>0.856443</v>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>6.6y Applied ML Engineer; hands-on embedding &amp; retrieval work at Sarvam AI; active GitHub (score 45); replies to 78% of recruiter messages. Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="42" customHeight="1">
       <c r="A45" t="inlineStr">
         <is>
           <t>CAND_0098846</t>
@@ -1227,16 +1237,16 @@
       <c r="B45" t="n">
         <v>44</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C45" s="2" t="n">
         <v>0.856365</v>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>AI Engineer with 7.6y: hands-on relevance &amp; ranking work at upGrad; decent recruiter response rate (0.62); open to relocation. Watch-out: ~70 days since last platform activity.</t>
         </is>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="42" customHeight="1">
       <c r="A46" t="inlineStr">
         <is>
           <t>CAND_0052335</t>
@@ -1245,16 +1255,16 @@
       <c r="B46" t="n">
         <v>45</v>
       </c>
-      <c r="C46" t="n">
+      <c r="C46" s="2" t="n">
         <v>0.854183</v>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>Applied ML Engineer, 6.4 yrs. Hands-on ranking &amp; embedding work at Aganitha; has evaluated rankers with NDCG/MRR/A-B testing; replies to 79% of recruiter messages. One flag: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="42" customHeight="1">
       <c r="A47" t="inlineStr">
         <is>
           <t>CAND_0052682</t>
@@ -1263,16 +1273,16 @@
       <c r="B47" t="n">
         <v>46</v>
       </c>
-      <c r="C47" t="n">
+      <c r="C47" s="2" t="n">
         <v>0.85253</v>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>NLP Engineer with 6.6y: hands-on embedding &amp; ranking work at Aganitha; replies to 88% of recruiter messages; can move on ~30-day notice. Watch-out: ~96 days since last platform activity.</t>
         </is>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="42" customHeight="1">
       <c r="A48" t="inlineStr">
         <is>
           <t>CAND_0058688</t>
@@ -1281,16 +1291,16 @@
       <c r="B48" t="n">
         <v>47</v>
       </c>
-      <c r="C48" t="n">
+      <c r="C48" s="2" t="n">
         <v>0.851473</v>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>AI Engineer, 6.7y: hands-on embedding &amp; ranking work at Vedantu; has evaluated rankers with NDCG/MRR/A-B testing; decent recruiter response rate (0.74). Concern: ~96 days since last platform activity.</t>
         </is>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="42" customHeight="1">
       <c r="A49" t="inlineStr">
         <is>
           <t>CAND_0079064</t>
@@ -1299,16 +1309,16 @@
       <c r="B49" t="n">
         <v>48</v>
       </c>
-      <c r="C49" t="n">
+      <c r="C49" s="2" t="n">
         <v>0.848484</v>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>Senior Data Scientist, 5.2y: hands-on semantic search &amp; retrieval work at Niramai; based in Noida; has evaluated rankers with NDCG/MRR/A-B testing. Concern: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="42" customHeight="1">
       <c r="A50" t="inlineStr">
         <is>
           <t>CAND_0088025</t>
@@ -1317,16 +1327,16 @@
       <c r="B50" t="n">
         <v>49</v>
       </c>
-      <c r="C50" t="n">
+      <c r="C50" s="2" t="n">
         <v>0.847164</v>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>8.6y Staff Machine Learning Engineer; hands-on recommend &amp; retrieval work at Yellow.ai; active GitHub (score 75); replies to 83% of recruiter messages. Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="42" customHeight="1">
       <c r="A51" t="inlineStr">
         <is>
           <t>CAND_0086151</t>
@@ -1335,16 +1345,16 @@
       <c r="B51" t="n">
         <v>50</v>
       </c>
-      <c r="C51" t="n">
+      <c r="C51" s="2" t="n">
         <v>0.846557</v>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>Recommendation Systems Engineer, 7.7 yrs. Hands-on retrieval &amp; ranking work at Wysa; Redrob assessment 84 in Recommendation Systems; has evaluated rankers with NDCG/MRR/A-B testing. One flag: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="52">
+    <row r="52" ht="42" customHeight="1">
       <c r="A52" t="inlineStr">
         <is>
           <t>CAND_0014440</t>
@@ -1353,16 +1363,16 @@
       <c r="B52" t="n">
         <v>51</v>
       </c>
-      <c r="C52" t="n">
+      <c r="C52" s="2" t="n">
         <v>0.844948</v>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>Recommendation Systems Engineer, 6.4y: hands-on recommend &amp; relevance work at CRED; decent recruiter response rate (0.64); based in Chennai. Concern: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="53">
+    <row r="53" ht="42" customHeight="1">
       <c r="A53" t="inlineStr">
         <is>
           <t>CAND_0091909</t>
@@ -1371,16 +1381,16 @@
       <c r="B53" t="n">
         <v>52</v>
       </c>
-      <c r="C53" t="n">
+      <c r="C53" s="2" t="n">
         <v>0.84426</v>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>6.9y Machine Learning Engineer; hands-on recommend &amp; embedding work at Rephrase.ai; Redrob assessment 90 in Image Classification; has evaluated rankers with NDCG/MRR/A-B testing. Main caveat: ~106 days since last platform activity.</t>
         </is>
       </c>
     </row>
-    <row r="54">
+    <row r="54" ht="42" customHeight="1">
       <c r="A54" t="inlineStr">
         <is>
           <t>CAND_0096142</t>
@@ -1389,16 +1399,16 @@
       <c r="B54" t="n">
         <v>53</v>
       </c>
-      <c r="C54" t="n">
+      <c r="C54" s="2" t="n">
         <v>0.8341229999999999</v>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>Applied ML Engineer with 5.0y: hands-on recommend &amp; embedding work at upGrad; replies to 84% of recruiter messages; based in Hyderabad. Watch-out: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="55">
+    <row r="55" ht="42" customHeight="1">
       <c r="A55" t="inlineStr">
         <is>
           <t>CAND_0017960</t>
@@ -1407,16 +1417,16 @@
       <c r="B55" t="n">
         <v>54</v>
       </c>
-      <c r="C55" t="n">
+      <c r="C55" s="2" t="n">
         <v>0.832237</v>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>Recommendation Systems Engineer, 7.7y: hands-on embedding &amp; ranking work at Nykaa; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 92). Concern: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="56">
+    <row r="56" ht="42" customHeight="1">
       <c r="A56" t="inlineStr">
         <is>
           <t>CAND_0012837</t>
@@ -1425,16 +1435,16 @@
       <c r="B56" t="n">
         <v>55</v>
       </c>
-      <c r="C56" t="n">
+      <c r="C56" s="2" t="n">
         <v>0.831021</v>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>6.4y Junior ML Engineer; hands-on ranking &amp; re-rank work at Sarvam AI; replies to 81% of recruiter messages; open to relocation. Main caveat: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="57">
+    <row r="57" ht="42" customHeight="1">
       <c r="A57" t="inlineStr">
         <is>
           <t>CAND_0048558</t>
@@ -1443,16 +1453,16 @@
       <c r="B57" t="n">
         <v>56</v>
       </c>
-      <c r="C57" t="n">
+      <c r="C57" s="2" t="n">
         <v>0.8292079999999999</v>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>Data Scientist with 6.7y: hands-on ranking &amp; re-rank work at Rephrase.ai; replies to 80% of recruiter messages; can move on ~30-day notice. Watch-out: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
-    <row r="58">
+    <row r="58" ht="42" customHeight="1">
       <c r="A58" t="inlineStr">
         <is>
           <t>CAND_0043228</t>
@@ -1461,16 +1471,16 @@
       <c r="B58" t="n">
         <v>57</v>
       </c>
-      <c r="C58" t="n">
+      <c r="C58" s="2" t="n">
         <v>0.825628</v>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Applied ML Engineer, 6.8y: hands-on ranking &amp; semantic search work at Zoho; active GitHub (score 48); can move on ~30-day notice. Concern: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
-    <row r="59">
+    <row r="59" ht="42" customHeight="1">
       <c r="A59" t="inlineStr">
         <is>
           <t>CAND_0010149</t>
@@ -1479,16 +1489,16 @@
       <c r="B59" t="n">
         <v>58</v>
       </c>
-      <c r="C59" t="n">
+      <c r="C59" s="2" t="n">
         <v>0.823282</v>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>6.9y ML Engineer; hands-on ranking &amp; re-rank work at Glance; replies to 82% of recruiter messages; based in Bangalore. Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="60">
+    <row r="60" ht="42" customHeight="1">
       <c r="A60" t="inlineStr">
         <is>
           <t>CAND_0094056</t>
@@ -1497,16 +1507,16 @@
       <c r="B60" t="n">
         <v>59</v>
       </c>
-      <c r="C60" t="n">
+      <c r="C60" s="2" t="n">
         <v>0.822871</v>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>NLP Engineer, 5.9y: hands-on retrieval &amp; recommend work at Rephrase.ai; active GitHub (score 65); replies to 82% of recruiter messages. Concern: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="42" customHeight="1">
       <c r="A61" t="inlineStr">
         <is>
           <t>CAND_0011327</t>
@@ -1515,16 +1525,16 @@
       <c r="B61" t="n">
         <v>60</v>
       </c>
-      <c r="C61" t="n">
+      <c r="C61" s="2" t="n">
         <v>0.820395</v>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>AI Research Engineer, 6.3 yrs. Hands-on recommend &amp; ranking work at Krutrim; replies to 79% of recruiter messages; based in Gurgaon. One flag: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="62">
+    <row r="62" ht="42" customHeight="1">
       <c r="A62" t="inlineStr">
         <is>
           <t>CAND_0078002</t>
@@ -1533,16 +1543,16 @@
       <c r="B62" t="n">
         <v>61</v>
       </c>
-      <c r="C62" t="n">
+      <c r="C62" s="2" t="n">
         <v>0.818458</v>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="3" t="inlineStr">
         <is>
           <t>Machine Learning Engineer with 6.3y: hands-on embedding &amp; ranking work at Meta; replies to 86% of recruiter messages; Redrob assessment 80 in pgvector. Watch-out: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="42" customHeight="1">
       <c r="A63" t="inlineStr">
         <is>
           <t>CAND_0018722</t>
@@ -1551,16 +1561,16 @@
       <c r="B63" t="n">
         <v>62</v>
       </c>
-      <c r="C63" t="n">
+      <c r="C63" s="2" t="n">
         <v>0.817858</v>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="3" t="inlineStr">
         <is>
           <t>Recommendation Systems Engineer with 6.6y: hands-on recommend &amp; retrieval work at Saarthi.ai; open to relocation; active GitHub (score 94). Watch-out: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="42" customHeight="1">
       <c r="A64" t="inlineStr">
         <is>
           <t>CAND_0051292</t>
@@ -1569,16 +1579,16 @@
       <c r="B64" t="n">
         <v>63</v>
       </c>
-      <c r="C64" t="n">
+      <c r="C64" s="2" t="n">
         <v>0.817778</v>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>Applied ML Engineer, 5.2y: hands-on ranking &amp; embedding work at Freshworks; active GitHub (score 62); can move on ~30-day notice. Concern: average stint is only ~20 months across 3 roles.</t>
         </is>
       </c>
     </row>
-    <row r="65">
+    <row r="65" ht="42" customHeight="1">
       <c r="A65" t="inlineStr">
         <is>
           <t>CAND_0049896</t>
@@ -1587,16 +1597,16 @@
       <c r="B65" t="n">
         <v>64</v>
       </c>
-      <c r="C65" t="n">
+      <c r="C65" s="2" t="n">
         <v>0.816051</v>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="3" t="inlineStr">
         <is>
           <t>Search Engineer, 7.3y: hands-on ranking &amp; recommend work at Unacademy; has evaluated rankers with NDCG/MRR/A-B testing; open to relocation. Concern: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="66">
+    <row r="66" ht="42" customHeight="1">
       <c r="A66" t="inlineStr">
         <is>
           <t>CAND_0039754</t>
@@ -1605,16 +1615,16 @@
       <c r="B66" t="n">
         <v>65</v>
       </c>
-      <c r="C66" t="n">
+      <c r="C66" s="2" t="n">
         <v>0.814277</v>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>Senior Applied Scientist with 16.2y: hands-on ranking &amp; re-rank work at Meta; open to relocation; Redrob assessment 96 in Fine-tuning LLMs. Watch-out: 16.2y experience falls outside the JD's 5-9y band.</t>
         </is>
       </c>
     </row>
-    <row r="67">
+    <row r="67" ht="42" customHeight="1">
       <c r="A67" t="inlineStr">
         <is>
           <t>CAND_0000031</t>
@@ -1623,16 +1633,16 @@
       <c r="B67" t="n">
         <v>66</v>
       </c>
-      <c r="C67" t="n">
+      <c r="C67" s="2" t="n">
         <v>0.813544</v>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D67" s="3" t="inlineStr">
         <is>
           <t>Recommendation Systems Engineer, 6.0 yrs. Hands-on recommend &amp; relevance work at Swiggy; Redrob assessment 75 in MLflow; has evaluated rankers with NDCG/MRR/A-B testing. One flag: average stint is only ~18 months across 4 roles.</t>
         </is>
       </c>
     </row>
-    <row r="68">
+    <row r="68" ht="42" customHeight="1">
       <c r="A68" t="inlineStr">
         <is>
           <t>CAND_0028793</t>
@@ -1641,16 +1651,16 @@
       <c r="B68" t="n">
         <v>67</v>
       </c>
-      <c r="C68" t="n">
+      <c r="C68" s="2" t="n">
         <v>0.811156</v>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr">
         <is>
           <t>7.2y Search Engineer; hands-on embedding &amp; retrieval work at Google; open to relocation; Redrob assessment 89 in Embeddings. Main caveat: 120-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="69">
+    <row r="69" ht="42" customHeight="1">
       <c r="A69" t="inlineStr">
         <is>
           <t>CAND_0033179</t>
@@ -1659,16 +1669,16 @@
       <c r="B69" t="n">
         <v>68</v>
       </c>
-      <c r="C69" t="n">
+      <c r="C69" s="2" t="n">
         <v>0.8107529999999999</v>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69" s="3" t="inlineStr">
         <is>
           <t>AI Research Engineer, 6.9 yrs. Hands-on recommend &amp; ranking work at Wipro; Redrob assessment 82 in Speech Recognition; replies to 84% of recruiter messages. One flag: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
-    <row r="70">
+    <row r="70" ht="42" customHeight="1">
       <c r="A70" t="inlineStr">
         <is>
           <t>CAND_0011432</t>
@@ -1677,16 +1687,16 @@
       <c r="B70" t="n">
         <v>69</v>
       </c>
-      <c r="C70" t="n">
+      <c r="C70" s="2" t="n">
         <v>0.810717</v>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D70" s="3" t="inlineStr">
         <is>
           <t>Senior Data Scientist, 7.6y: hands-on machine learning &amp; ranking work at Amazon; has evaluated rankers with NDCG/MRR/A-B testing; decent recruiter response rate (0.67). Concern: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="71">
+    <row r="71" ht="42" customHeight="1">
       <c r="A71" t="inlineStr">
         <is>
           <t>CAND_0095528</t>
@@ -1695,16 +1705,16 @@
       <c r="B71" t="n">
         <v>70</v>
       </c>
-      <c r="C71" t="n">
+      <c r="C71" s="2" t="n">
         <v>0.810427</v>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="D71" s="3" t="inlineStr">
         <is>
           <t>Senior Data Scientist, 5.3y: hands-on embedding &amp; ranking work at Netflix; Redrob assessment 87 in pgvector; has evaluated rankers with NDCG/MRR/A-B testing. Concern: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
-    <row r="72">
+    <row r="72" ht="42" customHeight="1">
       <c r="A72" t="inlineStr">
         <is>
           <t>CAND_0099401</t>
@@ -1713,16 +1723,16 @@
       <c r="B72" t="n">
         <v>71</v>
       </c>
-      <c r="C72" t="n">
+      <c r="C72" s="2" t="n">
         <v>0.8103359999999999</v>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D72" s="3" t="inlineStr">
         <is>
           <t>7.7y NLP Engineer; hands-on embedding &amp; ranking work at Dream11; has evaluated rankers with NDCG/MRR/A-B testing; open to relocation. Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="73">
+    <row r="73" ht="42" customHeight="1">
       <c r="A73" t="inlineStr">
         <is>
           <t>CAND_0042029</t>
@@ -1731,16 +1741,16 @@
       <c r="B73" t="n">
         <v>72</v>
       </c>
-      <c r="C73" t="n">
+      <c r="C73" s="2" t="n">
         <v>0.809364</v>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D73" s="3" t="inlineStr">
         <is>
           <t>6.5y Senior Data Scientist; hands-on machine learning &amp; ranking work at Flipkart; Redrob assessment 83 in YOLO; has evaluated rankers with NDCG/MRR/A-B testing. Main caveat: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
-    <row r="74">
+    <row r="74" ht="42" customHeight="1">
       <c r="A74" t="inlineStr">
         <is>
           <t>CAND_0002025</t>
@@ -1749,16 +1759,16 @@
       <c r="B74" t="n">
         <v>73</v>
       </c>
-      <c r="C74" t="n">
+      <c r="C74" s="2" t="n">
         <v>0.809131</v>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D74" s="3" t="inlineStr">
         <is>
           <t>5.9y Senior AI Engineer; hands-on ranking &amp; re-rank work at Apple; active GitHub (score 97); replies to 80% of recruiter messages. Main caveat: little to fault on paper; verify depth in a technical screen.</t>
         </is>
       </c>
     </row>
-    <row r="75">
+    <row r="75" ht="42" customHeight="1">
       <c r="A75" t="inlineStr">
         <is>
           <t>CAND_0047721</t>
@@ -1767,16 +1777,16 @@
       <c r="B75" t="n">
         <v>74</v>
       </c>
-      <c r="C75" t="n">
+      <c r="C75" s="2" t="n">
         <v>0.806061</v>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D75" s="3" t="inlineStr">
         <is>
           <t>7.0y Senior Data Scientist; hands-on ranking &amp; recommend work at Microsoft; active GitHub (score 90); open to relocation. Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="76">
+    <row r="76" ht="42" customHeight="1">
       <c r="A76" t="inlineStr">
         <is>
           <t>CAND_0030953</t>
@@ -1785,16 +1795,16 @@
       <c r="B76" t="n">
         <v>75</v>
       </c>
-      <c r="C76" t="n">
+      <c r="C76" s="2" t="n">
         <v>0.804835</v>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D76" s="3" t="inlineStr">
         <is>
           <t>7.8y Search Engineer; hands-on recommend &amp; retrieval work at Nykaa; decent recruiter response rate (0.63); based in Chennai. Main caveat: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
-    <row r="77">
+    <row r="77" ht="42" customHeight="1">
       <c r="A77" t="inlineStr">
         <is>
           <t>CAND_0072660</t>
@@ -1803,16 +1813,16 @@
       <c r="B77" t="n">
         <v>76</v>
       </c>
-      <c r="C77" t="n">
+      <c r="C77" s="2" t="n">
         <v>0.80276</v>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D77" s="3" t="inlineStr">
         <is>
           <t>Machine Learning Engineer, 7.1y: hands-on ranking &amp; relevance work at Unacademy; can move on ~30-day notice. Concern: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
-    <row r="78">
+    <row r="78" ht="42" customHeight="1">
       <c r="A78" t="inlineStr">
         <is>
           <t>CAND_0081053</t>
@@ -1821,16 +1831,16 @@
       <c r="B78" t="n">
         <v>77</v>
       </c>
-      <c r="C78" t="n">
+      <c r="C78" s="2" t="n">
         <v>0.802405</v>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D78" s="3" t="inlineStr">
         <is>
           <t>5.4y NLP Engineer; hands-on embedding &amp; ranking work at Glance; open to relocation; Redrob assessment 89 in QLoRA. Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="79">
+    <row r="79" ht="42" customHeight="1">
       <c r="A79" t="inlineStr">
         <is>
           <t>CAND_0006567</t>
@@ -1839,16 +1849,16 @@
       <c r="B79" t="n">
         <v>78</v>
       </c>
-      <c r="C79" t="n">
+      <c r="C79" s="2" t="n">
         <v>0.801091</v>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D79" s="3" t="inlineStr">
         <is>
           <t>Senior AI Engineer, 7.9 yrs. Hands-on ranking &amp; relevance work at Meta; Redrob assessment 90 in scikit-learn; has evaluated rankers with NDCG/MRR/A-B testing. One flag: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="80">
+    <row r="80" ht="42" customHeight="1">
       <c r="A80" t="inlineStr">
         <is>
           <t>CAND_0070202</t>
@@ -1857,16 +1867,16 @@
       <c r="B80" t="n">
         <v>79</v>
       </c>
-      <c r="C80" t="n">
+      <c r="C80" s="2" t="n">
         <v>0.800609</v>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D80" s="3" t="inlineStr">
         <is>
           <t>Machine Learning Engineer with 5.1y: hands-on embedding &amp; ranking work at BYJU'S; Redrob assessment 89 in Object Detection; has evaluated rankers with NDCG/MRR/A-B testing. Watch-out: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="81">
+    <row r="81" ht="42" customHeight="1">
       <c r="A81" t="inlineStr">
         <is>
           <t>CAND_0015528</t>
@@ -1875,16 +1885,16 @@
       <c r="B81" t="n">
         <v>80</v>
       </c>
-      <c r="C81" t="n">
+      <c r="C81" s="2" t="n">
         <v>0.800566</v>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D81" s="3" t="inlineStr">
         <is>
           <t>Applied ML Engineer, 7.4y: hands-on ranking &amp; recommend work at Krutrim; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 51). Concern: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
-    <row r="82">
+    <row r="82" ht="42" customHeight="1">
       <c r="A82" t="inlineStr">
         <is>
           <t>CAND_0050876</t>
@@ -1893,16 +1903,16 @@
       <c r="B82" t="n">
         <v>81</v>
       </c>
-      <c r="C82" t="n">
+      <c r="C82" s="2" t="n">
         <v>0.799821</v>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="D82" s="3" t="inlineStr">
         <is>
           <t>Applied ML Engineer, 6.0y: hands-on embedding &amp; ranking work at Freshworks; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 86). Concern: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="83">
+    <row r="83" ht="42" customHeight="1">
       <c r="A83" t="inlineStr">
         <is>
           <t>CAND_0093912</t>
@@ -1911,16 +1921,16 @@
       <c r="B83" t="n">
         <v>82</v>
       </c>
-      <c r="C83" t="n">
+      <c r="C83" s="2" t="n">
         <v>0.798781</v>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D83" s="3" t="inlineStr">
         <is>
           <t>Senior Data Scientist, 5.3y: hands-on retrieval &amp; ranking work at Razorpay; active GitHub (score 82); decent recruiter response rate (0.66). Concern: average stint is only ~21 months across 3 roles.</t>
         </is>
       </c>
     </row>
-    <row r="84">
+    <row r="84" ht="42" customHeight="1">
       <c r="A84" t="inlineStr">
         <is>
           <t>CAND_0061257</t>
@@ -1929,16 +1939,16 @@
       <c r="B84" t="n">
         <v>83</v>
       </c>
-      <c r="C84" t="n">
+      <c r="C84" s="2" t="n">
         <v>0.797652</v>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D84" s="3" t="inlineStr">
         <is>
           <t>8.0y Staff Machine Learning Engineer; hands-on ranking &amp; relevance work at LinkedIn; replies to 87% of recruiter messages; can move on ~30-day notice. Main caveat: ~77 days since last platform activity.</t>
         </is>
       </c>
     </row>
-    <row r="85">
+    <row r="85" ht="42" customHeight="1">
       <c r="A85" t="inlineStr">
         <is>
           <t>CAND_0026532</t>
@@ -1947,16 +1957,16 @@
       <c r="B85" t="n">
         <v>84</v>
       </c>
-      <c r="C85" t="n">
+      <c r="C85" s="2" t="n">
         <v>0.796786</v>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D85" s="3" t="inlineStr">
         <is>
           <t>Recommendation Systems Engineer, 4.8y: hands-on retrieval &amp; ranking work at Zomato; has evaluated rankers with NDCG/MRR/A-B testing; based in Chennai. Concern: 4.8y experience falls outside the JD's 5-9y band.</t>
         </is>
       </c>
     </row>
-    <row r="86">
+    <row r="86" ht="42" customHeight="1">
       <c r="A86" t="inlineStr">
         <is>
           <t>CAND_0042100</t>
@@ -1965,16 +1975,16 @@
       <c r="B86" t="n">
         <v>85</v>
       </c>
-      <c r="C86" t="n">
+      <c r="C86" s="2" t="n">
         <v>0.793462</v>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D86" s="3" t="inlineStr">
         <is>
           <t>Machine Learning Engineer, 7.3y: hands-on relevance &amp; machine learning work at Freshworks; has evaluated rankers with NDCG/MRR/A-B testing; active GitHub (score 43). Concern: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="87">
+    <row r="87" ht="42" customHeight="1">
       <c r="A87" t="inlineStr">
         <is>
           <t>CAND_0053527</t>
@@ -1983,16 +1993,16 @@
       <c r="B87" t="n">
         <v>86</v>
       </c>
-      <c r="C87" t="n">
+      <c r="C87" s="2" t="n">
         <v>0.792774</v>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D87" s="3" t="inlineStr">
         <is>
           <t>Junior ML Engineer, 7.0 yrs. Hands-on re-rank &amp; recommend work at PhonePe; replies to 81% of recruiter messages; based in Bangalore. One flag: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="88">
+    <row r="88" ht="42" customHeight="1">
       <c r="A88" t="inlineStr">
         <is>
           <t>CAND_0016659</t>
@@ -2001,16 +2011,16 @@
       <c r="B88" t="n">
         <v>87</v>
       </c>
-      <c r="C88" t="n">
+      <c r="C88" s="2" t="n">
         <v>0.784655</v>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D88" s="3" t="inlineStr">
         <is>
           <t>ML Engineer, 4.4 yrs. Hands-on ranking &amp; re-rank work at Glance; replies to 89% of recruiter messages; Redrob assessment 78 in Information Retrieval. One flag: 4.4y experience falls outside the JD's 5-9y band.</t>
         </is>
       </c>
     </row>
-    <row r="89">
+    <row r="89" ht="42" customHeight="1">
       <c r="A89" t="inlineStr">
         <is>
           <t>CAND_0066999</t>
@@ -2019,16 +2029,16 @@
       <c r="B89" t="n">
         <v>88</v>
       </c>
-      <c r="C89" t="n">
+      <c r="C89" s="2" t="n">
         <v>0.784573</v>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D89" s="3" t="inlineStr">
         <is>
           <t>Recommendation Systems Engineer, 5.9 yrs. Hands-on ranking &amp; recommend work at Microsoft; Redrob assessment 90 in Pinecone; active GitHub (score 94). One flag: ~88 days since last platform activity.</t>
         </is>
       </c>
     </row>
-    <row r="90">
+    <row r="90" ht="42" customHeight="1">
       <c r="A90" t="inlineStr">
         <is>
           <t>CAND_0031593</t>
@@ -2037,16 +2047,16 @@
       <c r="B90" t="n">
         <v>89</v>
       </c>
-      <c r="C90" t="n">
+      <c r="C90" s="2" t="n">
         <v>0.78334</v>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D90" s="3" t="inlineStr">
         <is>
           <t>7.8y Search Engineer; hands-on ranking &amp; recommend work at Genpact AI; has evaluated rankers with NDCG/MRR/A-B testing; decent recruiter response rate (0.58). Main caveat: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="91">
+    <row r="91" ht="42" customHeight="1">
       <c r="A91" t="inlineStr">
         <is>
           <t>CAND_0076163</t>
@@ -2055,16 +2065,16 @@
       <c r="B91" t="n">
         <v>90</v>
       </c>
-      <c r="C91" t="n">
+      <c r="C91" s="2" t="n">
         <v>0.783179</v>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D91" s="3" t="inlineStr">
         <is>
           <t>NLP Engineer, 6.9 yrs. Hands-on nlp &amp; ranking work at Ola; Redrob assessment 92 in BM25; active GitHub (score 85). One flag: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="92">
+    <row r="92" ht="42" customHeight="1">
       <c r="A92" t="inlineStr">
         <is>
           <t>CAND_0044262</t>
@@ -2073,16 +2083,16 @@
       <c r="B92" t="n">
         <v>91</v>
       </c>
-      <c r="C92" t="n">
+      <c r="C92" s="2" t="n">
         <v>0.7830780000000001</v>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="D92" s="3" t="inlineStr">
         <is>
           <t>Data Scientist with 6.9y: hands-on ranking &amp; re-rank work at upGrad; decent recruiter response rate (0.73); open to relocation. Watch-out: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="93">
+    <row r="93" ht="42" customHeight="1">
       <c r="A93" t="inlineStr">
         <is>
           <t>CAND_0075574</t>
@@ -2091,16 +2101,16 @@
       <c r="B93" t="n">
         <v>92</v>
       </c>
-      <c r="C93" t="n">
+      <c r="C93" s="2" t="n">
         <v>0.7812750000000001</v>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D93" s="3" t="inlineStr">
         <is>
           <t>Machine Learning Engineer with 5.7y: hands-on embedding &amp; relevance work at Haptik; based in Bangalore; Redrob assessment 83 in pgvector. Watch-out: 60-day notice needs a partial buyout.</t>
         </is>
       </c>
     </row>
-    <row r="94">
+    <row r="94" ht="42" customHeight="1">
       <c r="A94" t="inlineStr">
         <is>
           <t>CAND_0061655</t>
@@ -2109,16 +2119,16 @@
       <c r="B94" t="n">
         <v>93</v>
       </c>
-      <c r="C94" t="n">
+      <c r="C94" s="2" t="n">
         <v>0.78067</v>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D94" s="3" t="inlineStr">
         <is>
           <t>Machine Learning Engineer, 4.6 yrs. Hands-on embedding &amp; ranking work at Krutrim; can move on ~15-day notice; has evaluated rankers with NDCG/MRR/A-B testing. One flag: 4.6y experience falls outside the JD's 5-9y band.</t>
         </is>
       </c>
     </row>
-    <row r="95">
+    <row r="95" ht="42" customHeight="1">
       <c r="A95" t="inlineStr">
         <is>
           <t>CAND_0051630</t>
@@ -2127,16 +2137,16 @@
       <c r="B95" t="n">
         <v>94</v>
       </c>
-      <c r="C95" t="n">
+      <c r="C95" s="2" t="n">
         <v>0.780481</v>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D95" s="3" t="inlineStr">
         <is>
           <t>Machine Learning Engineer with 6.0y: hands-on retrieval &amp; ranking work at Razorpay; active GitHub (score 66). Watch-out: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="96">
+    <row r="96" ht="42" customHeight="1">
       <c r="A96" t="inlineStr">
         <is>
           <t>CAND_0080766</t>
@@ -2145,16 +2155,16 @@
       <c r="B96" t="n">
         <v>95</v>
       </c>
-      <c r="C96" t="n">
+      <c r="C96" s="2" t="n">
         <v>0.780443</v>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D96" s="3" t="inlineStr">
         <is>
           <t>Staff Machine Learning Engineer with 8.8y: hands-on retrieval &amp; ranking work at Salesforce; decent recruiter response rate (0.66); can move on ~0-day notice. Watch-out: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
-    <row r="97">
+    <row r="97" ht="42" customHeight="1">
       <c r="A97" t="inlineStr">
         <is>
           <t>CAND_0040178</t>
@@ -2163,16 +2173,16 @@
       <c r="B97" t="n">
         <v>96</v>
       </c>
-      <c r="C97" t="n">
+      <c r="C97" s="2" t="n">
         <v>0.7794759999999999</v>
       </c>
-      <c r="D97" t="inlineStr">
+      <c r="D97" s="3" t="inlineStr">
         <is>
           <t>ML Engineer with 5.0y: hands-on recommend &amp; ranking work at Meesho; decent recruiter response rate (0.55); based in Pune. Watch-out: average stint is only ~20 months across 3 roles.</t>
         </is>
       </c>
     </row>
-    <row r="98">
+    <row r="98" ht="42" customHeight="1">
       <c r="A98" t="inlineStr">
         <is>
           <t>CAND_0029367</t>
@@ -2181,16 +2191,16 @@
       <c r="B98" t="n">
         <v>97</v>
       </c>
-      <c r="C98" t="n">
+      <c r="C98" s="2" t="n">
         <v>0.779154</v>
       </c>
-      <c r="D98" t="inlineStr">
+      <c r="D98" s="3" t="inlineStr">
         <is>
           <t>Senior Data Scientist, 5.7 yrs. Hands-on retrieval &amp; embedding work at Rephrase.ai; Redrob assessment 90 in Haystack; has evaluated rankers with NDCG/MRR/A-B testing. One flag: 90-day notice period raises the bar per the JD.</t>
         </is>
       </c>
     </row>
-    <row r="99">
+    <row r="99" ht="42" customHeight="1">
       <c r="A99" t="inlineStr">
         <is>
           <t>CAND_0040117</t>
@@ -2199,16 +2209,16 @@
       <c r="B99" t="n">
         <v>98</v>
       </c>
-      <c r="C99" t="n">
+      <c r="C99" s="2" t="n">
         <v>0.778189</v>
       </c>
-      <c r="D99" t="inlineStr">
+      <c r="D99" s="3" t="inlineStr">
         <is>
           <t>6.5y Recommendation Systems Engineer; hands-on recommend &amp; embedding work at PhonePe; decent recruiter response rate (0.66); can move on ~15-day notice. Main caveat: no GitHub linked, so code activity cannot be verified.</t>
         </is>
       </c>
     </row>
-    <row r="100">
+    <row r="100" ht="42" customHeight="1">
       <c r="A100" t="inlineStr">
         <is>
           <t>CAND_0096172</t>
@@ -2217,16 +2227,16 @@
       <c r="B100" t="n">
         <v>99</v>
       </c>
-      <c r="C100" t="n">
+      <c r="C100" s="2" t="n">
         <v>0.777152</v>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="D100" s="3" t="inlineStr">
         <is>
           <t>NLP Engineer, 5.2y: hands-on ranking &amp; recommend work at Krutrim; active GitHub (score 65); based in Chennai. Concern: has not flagged themselves open to work.</t>
         </is>
       </c>
     </row>
-    <row r="101">
+    <row r="101" ht="42" customHeight="1">
       <c r="A101" t="inlineStr">
         <is>
           <t>CAND_0087630</t>
@@ -2235,10 +2245,10 @@
       <c r="B101" t="n">
         <v>100</v>
       </c>
-      <c r="C101" t="n">
+      <c r="C101" s="2" t="n">
         <v>0.776003</v>
       </c>
-      <c r="D101" t="inlineStr">
+      <c r="D101" s="3" t="inlineStr">
         <is>
           <t>AI Engineer with 7.2y: hands-on ranking &amp; recommend work at Vedantu; based in Gurgaon; Redrob assessment 78 in pgvector. Watch-out: has not flagged themselves open to work.</t>
         </is>

</xml_diff>